<commit_message>
Regenerate the SE packages and the advanced reconciliation report
The renumbered SE Full sheet flows into every generated year's
Financialaccounts.xlsx. The advanced scenario reconciles 678/678 with the
reworked checks.
</commit_message>
<xml_diff>
--- a/packages/GB Accounts Self Employed 2021-04-05 (Apr21) Excel 2007/Financialaccounts.xlsx
+++ b/packages/GB Accounts Self Employed 2021-04-05 (Apr21) Excel 2007/Financialaccounts.xlsx
@@ -7447,8 +7447,10 @@
         <v>10</v>
       </c>
       <c r="B36" s="181"/>
-      <c r="C36" s="182" t="s">
-        <v>167</v>
+      <c r="C36" s="182" t="inlineStr">
+        <is>
+          <t>If you used traditional accounting rather than cash basis to</t>
+        </is>
       </c>
       <c r="D36" s="182"/>
       <c r="E36" s="182"/>
@@ -7459,11 +7461,13 @@
       <c r="J36" s="182"/>
       <c r="K36" s="182"/>
       <c r="L36" s="194">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M36" s="181"/>
-      <c r="N36" s="182" t="s">
-        <v>168</v>
+      <c r="N36" s="182" t="inlineStr">
+        <is>
+          <t>If special arrangements apply, put 'X' in the box - read the</t>
+        </is>
       </c>
       <c r="O36" s="182"/>
       <c r="P36" s="182"/>
@@ -7478,8 +7482,10 @@
     <row r="37" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A37" s="185"/>
       <c r="B37" s="181"/>
-      <c r="C37" s="182" t="s">
-        <v>169</v>
+      <c r="C37" s="182" t="inlineStr">
+        <is>
+          <t>calculate your income and expenses, put 'X' in the box</t>
+        </is>
       </c>
       <c r="D37" s="182"/>
       <c r="E37" s="182"/>
@@ -7491,8 +7497,10 @@
       <c r="K37" s="182"/>
       <c r="L37" s="181"/>
       <c r="M37" s="181"/>
-      <c r="N37" s="182" t="s">
-        <v>170</v>
+      <c r="N37" s="182" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
       </c>
       <c r="O37" s="182"/>
       <c r="P37" s="182"/>
@@ -7580,12 +7588,12 @@
       <c r="W40" s="197"/>
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.15">
-      <c r="A41" s="194">
-        <v>11</v>
-      </c>
+      <c r="A41" s="194"/>
       <c r="B41" s="181"/>
-      <c r="C41" s="182" t="s">
-        <v>171</v>
+      <c r="C41" s="182" t="inlineStr">
+        <is>
+          <t>Boxes 11 and 12 are not in use</t>
+        </is>
       </c>
       <c r="D41" s="182"/>
       <c r="E41" s="182"/>
@@ -7596,7 +7604,7 @@
       <c r="J41" s="182"/>
       <c r="K41" s="182"/>
       <c r="L41" s="194">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M41" s="181"/>
       <c r="N41" s="182" t="str">
@@ -7616,9 +7624,7 @@
     <row r="42" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A42" s="185"/>
       <c r="B42" s="181"/>
-      <c r="C42" s="182" t="s">
-        <v>173</v>
-      </c>
+      <c r="C42" s="182"/>
       <c r="D42" s="182"/>
       <c r="E42" s="182"/>
       <c r="F42" s="182"/>
@@ -7629,8 +7635,10 @@
       <c r="K42" s="182"/>
       <c r="L42" s="181"/>
       <c r="M42" s="181"/>
-      <c r="N42" s="182" t="s">
-        <v>174</v>
+      <c r="N42" s="182" t="inlineStr">
+        <is>
+          <t>profit on last year's Tax Return put 'X' in the box</t>
+        </is>
       </c>
       <c r="O42" s="182"/>
       <c r="P42" s="182"/>
@@ -7656,9 +7664,7 @@
       <c r="K43" s="181"/>
       <c r="L43" s="181"/>
       <c r="M43" s="181"/>
-      <c r="N43" s="182" t="s">
-        <v>170</v>
-      </c>
+      <c r="N43" s="182"/>
       <c r="O43" s="182"/>
       <c r="P43" s="182"/>
       <c r="Q43" s="182"/>
@@ -13107,8 +13113,10 @@
         <v>5</v>
       </c>
       <c r="M14" s="220"/>
-      <c r="N14" s="227" t="s">
-        <v>150</v>
+      <c r="N14" s="227" t="inlineStr">
+        <is>
+          <t>If the details in boxes 1, 2, 3 or 4 have changed in the last 12</t>
+        </is>
       </c>
       <c r="O14" s="227"/>
       <c r="P14" s="227"/>
@@ -13137,8 +13145,10 @@
       <c r="K15" s="220"/>
       <c r="L15" s="220"/>
       <c r="M15" s="220"/>
-      <c r="N15" s="241" t="s">
-        <v>151</v>
+      <c r="N15" s="241" t="inlineStr">
+        <is>
+          <t>months, put 'X' in the box and give details in the 'Any other</t>
+        </is>
       </c>
       <c r="O15" s="227"/>
       <c r="P15" s="227"/>
@@ -13164,8 +13174,10 @@
       <c r="K16" s="220"/>
       <c r="L16" s="220"/>
       <c r="M16" s="220"/>
-      <c r="N16" s="227" t="s">
-        <v>152</v>
+      <c r="N16" s="227" t="inlineStr">
+        <is>
+          <t>information' box</t>
+        </is>
       </c>
       <c r="O16" s="268"/>
       <c r="P16" s="268"/>
@@ -13621,8 +13633,10 @@
         <v>4</v>
       </c>
       <c r="B32" s="220"/>
-      <c r="C32" s="241" t="s">
-        <v>162</v>
+      <c r="C32" s="241" t="inlineStr">
+        <is>
+          <t>Postcode of your business address</t>
+        </is>
       </c>
       <c r="D32" s="227"/>
       <c r="E32" s="227"/>
@@ -13669,8 +13683,10 @@
       <c r="K33" s="220"/>
       <c r="L33" s="220"/>
       <c r="M33" s="220"/>
-      <c r="N33" s="227" t="s">
-        <v>164</v>
+      <c r="N33" s="227" t="inlineStr">
+        <is>
+          <t>of your accounting period - read the notes if you have</t>
+        </is>
       </c>
       <c r="O33" s="227"/>
       <c r="P33" s="227"/>
@@ -13696,8 +13712,10 @@
       <c r="K34" s="220"/>
       <c r="L34" s="220"/>
       <c r="M34" s="220"/>
-      <c r="N34" s="246" t="s">
-        <v>165</v>
+      <c r="N34" s="246" t="inlineStr">
+        <is>
+          <t>filled in box 6 or 7</t>
+        </is>
       </c>
       <c r="O34" s="246"/>
       <c r="P34" s="227"/>
@@ -13819,8 +13837,10 @@
         <v>10</v>
       </c>
       <c r="B39" s="220"/>
-      <c r="C39" s="227" t="s">
-        <v>167</v>
+      <c r="C39" s="227" t="inlineStr">
+        <is>
+          <t>If you used traditional accounting rather than cash basis to</t>
+        </is>
       </c>
       <c r="D39" s="227"/>
       <c r="E39" s="227"/>
@@ -13831,11 +13851,13 @@
       <c r="J39" s="227"/>
       <c r="K39" s="227"/>
       <c r="L39" s="236">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M39" s="220"/>
-      <c r="N39" s="227" t="s">
-        <v>168</v>
+      <c r="N39" s="227" t="inlineStr">
+        <is>
+          <t>If special arrangements apply, put 'X' in the box - read the</t>
+        </is>
       </c>
       <c r="O39" s="227"/>
       <c r="P39" s="227"/>
@@ -13850,8 +13872,10 @@
     <row r="40" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A40" s="240"/>
       <c r="B40" s="220"/>
-      <c r="C40" s="227" t="s">
-        <v>169</v>
+      <c r="C40" s="227" t="inlineStr">
+        <is>
+          <t>calculate your income and expenses, put 'X' in the box</t>
+        </is>
       </c>
       <c r="D40" s="227"/>
       <c r="E40" s="227"/>
@@ -13863,8 +13887,10 @@
       <c r="K40" s="227"/>
       <c r="L40" s="220"/>
       <c r="M40" s="220"/>
-      <c r="N40" s="227" t="s">
-        <v>170</v>
+      <c r="N40" s="227" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
       </c>
       <c r="O40" s="227"/>
       <c r="P40" s="227"/>
@@ -13958,12 +13984,12 @@
       <c r="W43" s="243"/>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.15">
-      <c r="A44" s="236">
-        <v>11</v>
-      </c>
+      <c r="A44" s="236"/>
       <c r="B44" s="220"/>
-      <c r="C44" s="227" t="s">
-        <v>171</v>
+      <c r="C44" s="227" t="inlineStr">
+        <is>
+          <t>Boxes 11 and 12 are not in use</t>
+        </is>
       </c>
       <c r="D44" s="227"/>
       <c r="E44" s="227"/>
@@ -13974,11 +14000,12 @@
       <c r="J44" s="227"/>
       <c r="K44" s="227"/>
       <c r="L44" s="236">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M44" s="220"/>
-      <c r="N44" s="227" t="s">
-        <v>172</v>
+      <c r="N44" s="227" t="str">
+        <f>"If you provided the information about your "&amp;Admin!G2</f>
+        <v>If you provided the information about your 2025-26</v>
       </c>
       <c r="O44" s="227"/>
       <c r="P44" s="227"/>
@@ -13993,9 +14020,7 @@
     <row r="45" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A45" s="240"/>
       <c r="B45" s="220"/>
-      <c r="C45" s="227" t="s">
-        <v>173</v>
-      </c>
+      <c r="C45" s="227"/>
       <c r="D45" s="227"/>
       <c r="E45" s="227"/>
       <c r="F45" s="227"/>
@@ -14006,8 +14031,10 @@
       <c r="K45" s="227"/>
       <c r="L45" s="220"/>
       <c r="M45" s="220"/>
-      <c r="N45" s="227" t="s">
-        <v>174</v>
+      <c r="N45" s="227" t="inlineStr">
+        <is>
+          <t>profit on last year's tax return, put 'X' in the box</t>
+        </is>
       </c>
       <c r="O45" s="227"/>
       <c r="P45" s="227"/>
@@ -14033,9 +14060,7 @@
       <c r="K46" s="220"/>
       <c r="L46" s="220"/>
       <c r="M46" s="220"/>
-      <c r="N46" s="227" t="s">
-        <v>170</v>
-      </c>
+      <c r="N46" s="227"/>
       <c r="O46" s="227"/>
       <c r="P46" s="227"/>
       <c r="Q46" s="227"/>
@@ -14074,10 +14099,7 @@
     <row r="48" spans="1:23" ht="14" x14ac:dyDescent="0.15">
       <c r="A48" s="240"/>
       <c r="B48" s="220"/>
-      <c r="C48" s="272" t="str">
-        <f>IF('Business Details'!C45="x","x"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
+      <c r="C48" s="272"/>
       <c r="D48" s="220"/>
       <c r="E48" s="220"/>
       <c r="F48" s="220"/>
@@ -14181,7 +14203,7 @@
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A52" s="236">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B52" s="220"/>
       <c r="C52" s="227" t="s">
@@ -14196,11 +14218,13 @@
       <c r="J52" s="227"/>
       <c r="K52" s="227"/>
       <c r="L52" s="236">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M52" s="220"/>
-      <c r="N52" s="227" t="s">
-        <v>188</v>
+      <c r="N52" s="227" t="inlineStr">
+        <is>
+          <t>Any other business income not included in box 15</t>
+        </is>
       </c>
       <c r="O52" s="227"/>
       <c r="P52" s="227"/>
@@ -14228,9 +14252,7 @@
       <c r="K53" s="220"/>
       <c r="L53" s="220"/>
       <c r="M53" s="220"/>
-      <c r="N53" s="246" t="s">
-        <v>190</v>
-      </c>
+      <c r="N53" s="246"/>
       <c r="O53" s="220"/>
       <c r="P53" s="220"/>
       <c r="Q53" s="220"/>
@@ -14366,8 +14388,10 @@
       <c r="W57" s="365"/>
     </row>
     <row r="58" spans="1:23" s="254" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A58" s="366" t="s">
-        <v>192</v>
+      <c r="A58" s="366" t="inlineStr">
+        <is>
+          <t>Please read the 'Self-employment (full) notes' before filling in this section.</t>
+        </is>
       </c>
       <c r="B58" s="366"/>
       <c r="C58" s="366"/>
@@ -14449,8 +14473,10 @@
     <row r="61" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A61" s="240"/>
       <c r="B61" s="220"/>
-      <c r="C61" s="227" t="s">
-        <v>193</v>
+      <c r="C61" s="227" t="inlineStr">
+        <is>
+          <t>If your annual turnover was below £90,000, you may</t>
+        </is>
       </c>
       <c r="D61" s="227"/>
       <c r="E61" s="227"/>
@@ -14462,8 +14488,10 @@
       <c r="K61" s="227"/>
       <c r="L61" s="227"/>
       <c r="M61" s="227"/>
-      <c r="N61" s="227" t="s">
-        <v>194</v>
+      <c r="N61" s="227" t="inlineStr">
+        <is>
+          <t>Use this column if the figures in boxes 17 to 30</t>
+        </is>
       </c>
       <c r="O61" s="227"/>
       <c r="P61" s="227"/>
@@ -14478,8 +14506,10 @@
     <row r="62" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A62" s="240"/>
       <c r="B62" s="220"/>
-      <c r="C62" s="227" t="s">
-        <v>195</v>
+      <c r="C62" s="227" t="inlineStr">
+        <is>
+          <t>just put your total expenses in box 31</t>
+        </is>
       </c>
       <c r="D62" s="227"/>
       <c r="E62" s="227"/>
@@ -14531,11 +14561,13 @@
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A64" s="236">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B64" s="220"/>
-      <c r="C64" s="227" t="s">
-        <v>197</v>
+      <c r="C64" s="227" t="inlineStr">
+        <is>
+          <t>Cost of goods bought for resale or goods used</t>
+        </is>
       </c>
       <c r="D64" s="227"/>
       <c r="E64" s="227"/>
@@ -14546,7 +14578,7 @@
       <c r="J64" s="227"/>
       <c r="K64" s="227"/>
       <c r="L64" s="236">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M64" s="220"/>
       <c r="N64" s="220"/>
@@ -14656,7 +14688,7 @@
     </row>
     <row r="68" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A68" s="236">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B68" s="220"/>
       <c r="C68" s="227" t="s">
@@ -14671,7 +14703,7 @@
       <c r="J68" s="227"/>
       <c r="K68" s="227"/>
       <c r="L68" s="236">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M68" s="220"/>
       <c r="N68" s="220"/>
@@ -14781,7 +14813,7 @@
     </row>
     <row r="72" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A72" s="236">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B72" s="220"/>
       <c r="C72" s="227" t="s">
@@ -14796,7 +14828,7 @@
       <c r="J72" s="227"/>
       <c r="K72" s="227"/>
       <c r="L72" s="236">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M72" s="220"/>
       <c r="N72" s="220"/>
@@ -14906,11 +14938,13 @@
     </row>
     <row r="76" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A76" s="236">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B76" s="220"/>
-      <c r="C76" s="227" t="s">
-        <v>200</v>
+      <c r="C76" s="227" t="inlineStr">
+        <is>
+          <t>Car, van and travel expenses</t>
+        </is>
       </c>
       <c r="D76" s="227"/>
       <c r="E76" s="227"/>
@@ -14921,7 +14955,7 @@
       <c r="J76" s="227"/>
       <c r="K76" s="227"/>
       <c r="L76" s="236">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M76" s="220"/>
       <c r="N76" s="220"/>
@@ -15031,7 +15065,7 @@
     </row>
     <row r="80" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A80" s="236">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B80" s="220"/>
       <c r="C80" s="227" t="s">
@@ -15046,7 +15080,7 @@
       <c r="J80" s="227"/>
       <c r="K80" s="227"/>
       <c r="L80" s="236">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M80" s="220"/>
       <c r="N80" s="220"/>
@@ -15156,11 +15190,13 @@
     </row>
     <row r="84" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A84" s="236">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B84" s="220"/>
-      <c r="C84" s="227" t="s">
-        <v>202</v>
+      <c r="C84" s="227" t="inlineStr">
+        <is>
+          <t>Repairs and maintenance of property and equipment</t>
+        </is>
       </c>
       <c r="D84" s="227"/>
       <c r="E84" s="227"/>
@@ -15171,7 +15207,7 @@
       <c r="J84" s="227"/>
       <c r="K84" s="227"/>
       <c r="L84" s="236">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M84" s="220"/>
       <c r="N84" s="220"/>
@@ -15281,11 +15317,13 @@
     </row>
     <row r="88" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A88" s="236">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B88" s="220"/>
-      <c r="C88" s="227" t="s">
-        <v>203</v>
+      <c r="C88" s="227" t="inlineStr">
+        <is>
+          <t>Phone, fax, stationery and other office costs</t>
+        </is>
       </c>
       <c r="D88" s="227"/>
       <c r="E88" s="227"/>
@@ -15296,7 +15334,7 @@
       <c r="J88" s="227"/>
       <c r="K88" s="227"/>
       <c r="L88" s="236">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M88" s="220"/>
       <c r="N88" s="220"/>
@@ -15406,7 +15444,7 @@
     </row>
     <row r="92" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A92" s="236">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B92" s="220"/>
       <c r="C92" s="227" t="s">
@@ -15421,7 +15459,7 @@
       <c r="J92" s="227"/>
       <c r="K92" s="227"/>
       <c r="L92" s="236">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M92" s="220"/>
       <c r="N92" s="220"/>
@@ -15531,7 +15569,7 @@
     </row>
     <row r="96" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A96" s="236">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B96" s="220"/>
       <c r="C96" s="227" t="s">
@@ -15546,7 +15584,7 @@
       <c r="J96" s="227"/>
       <c r="K96" s="227"/>
       <c r="L96" s="236">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M96" s="220"/>
       <c r="N96" s="220"/>
@@ -15656,7 +15694,7 @@
     </row>
     <row r="100" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A100" s="236">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B100" s="220"/>
       <c r="C100" s="227" t="s">
@@ -15671,7 +15709,7 @@
       <c r="J100" s="227"/>
       <c r="K100" s="227"/>
       <c r="L100" s="236">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M100" s="220"/>
       <c r="N100" s="220"/>
@@ -15781,7 +15819,7 @@
     </row>
     <row r="104" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A104" s="236">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B104" s="220"/>
       <c r="C104" s="227" t="s">
@@ -15796,7 +15834,7 @@
       <c r="J104" s="227"/>
       <c r="K104" s="227"/>
       <c r="L104" s="236">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M104" s="220"/>
       <c r="N104" s="220"/>
@@ -15906,7 +15944,7 @@
     </row>
     <row r="108" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A108" s="236">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B108" s="220"/>
       <c r="C108" s="227" t="s">
@@ -15921,7 +15959,7 @@
       <c r="J108" s="227"/>
       <c r="K108" s="227"/>
       <c r="L108" s="236">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M108" s="220"/>
       <c r="N108" s="220"/>
@@ -16031,11 +16069,13 @@
     </row>
     <row r="112" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A112" s="236">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B112" s="220"/>
-      <c r="C112" s="227" t="s">
-        <v>209</v>
+      <c r="C112" s="227" t="inlineStr">
+        <is>
+          <t>Depreciation and loss or profit on sale of assets</t>
+        </is>
       </c>
       <c r="D112" s="227"/>
       <c r="E112" s="227"/>
@@ -16046,7 +16086,7 @@
       <c r="J112" s="227"/>
       <c r="K112" s="227"/>
       <c r="L112" s="236">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="M112" s="220"/>
       <c r="N112" s="220"/>
@@ -16159,7 +16199,7 @@
     </row>
     <row r="116" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A116" s="236">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B116" s="220"/>
       <c r="C116" s="227" t="s">
@@ -16174,7 +16214,7 @@
       <c r="J116" s="227"/>
       <c r="K116" s="227"/>
       <c r="L116" s="236">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M116" s="220"/>
       <c r="N116" s="220"/>
@@ -16284,11 +16324,13 @@
     </row>
     <row r="120" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A120" s="236">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B120" s="220"/>
-      <c r="C120" s="227" t="s">
-        <v>211</v>
+      <c r="C120" s="227" t="inlineStr">
+        <is>
+          <t>Total expenses (total of boxes 17 to 30)</t>
+        </is>
       </c>
       <c r="D120" s="227"/>
       <c r="E120" s="227"/>
@@ -16299,11 +16341,13 @@
       <c r="J120" s="227"/>
       <c r="K120" s="227"/>
       <c r="L120" s="236">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M120" s="220"/>
-      <c r="N120" s="227" t="s">
-        <v>212</v>
+      <c r="N120" s="227" t="inlineStr">
+        <is>
+          <t>Total disallowable expenses (total of boxes 32 to 45)</t>
+        </is>
       </c>
       <c r="O120" s="220"/>
       <c r="P120" s="220"/>
@@ -16466,7 +16510,7 @@
     </row>
     <row r="126" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A126" s="236">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B126" s="220"/>
       <c r="C126" s="227" t="s">
@@ -16481,11 +16525,13 @@
       <c r="J126" s="227"/>
       <c r="K126" s="227"/>
       <c r="L126" s="236">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M126" s="220"/>
-      <c r="N126" s="227" t="s">
-        <v>215</v>
+      <c r="N126" s="227" t="inlineStr">
+        <is>
+          <t>Or, net loss - if your expenses are more than your</t>
+        </is>
       </c>
       <c r="O126" s="220"/>
       <c r="P126" s="220"/>
@@ -16500,8 +16546,10 @@
     <row r="127" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A127" s="240"/>
       <c r="B127" s="220"/>
-      <c r="C127" s="246" t="s">
-        <v>216</v>
+      <c r="C127" s="246" t="inlineStr">
+        <is>
+          <t>expenses (if box 15 + box 16 minus box 31 is positive)</t>
+        </is>
       </c>
       <c r="D127" s="227"/>
       <c r="E127" s="227"/>
@@ -16513,8 +16561,10 @@
       <c r="K127" s="227"/>
       <c r="L127" s="220"/>
       <c r="M127" s="220"/>
-      <c r="N127" s="227" t="s">
-        <v>217</v>
+      <c r="N127" s="227" t="inlineStr">
+        <is>
+          <t>business income (if box 31 minus (box 15 + box 16) is positive)</t>
+        </is>
       </c>
       <c r="O127" s="220"/>
       <c r="P127" s="220"/>
@@ -16651,8 +16701,10 @@
       <c r="W131" s="365"/>
     </row>
     <row r="132" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A132" s="366" t="s">
-        <v>219</v>
+      <c r="A132" s="366" t="inlineStr">
+        <is>
+          <t>There are 'capital' tax allowances for vehicles, equipment and certain buildings used in your business (do not include the cost</t>
+        </is>
       </c>
       <c r="B132" s="366"/>
       <c r="C132" s="366"/>
@@ -16678,8 +16730,10 @@
       <c r="W132" s="366"/>
     </row>
     <row r="133" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A133" s="366" t="s">
-        <v>352</v>
+      <c r="A133" s="366" t="inlineStr">
+        <is>
+          <t>of these in your business expenses). Please read the 'Self-employment (full) notes' and use the examples to work out your</t>
+        </is>
       </c>
       <c r="B133" s="366"/>
       <c r="C133" s="366"/>
@@ -16705,8 +16759,10 @@
       <c r="W133" s="366"/>
     </row>
     <row r="134" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A134" s="366" t="s">
-        <v>220</v>
+      <c r="A134" s="366" t="inlineStr">
+        <is>
+          <t>capital allowances.</t>
+        </is>
       </c>
       <c r="B134" s="366"/>
       <c r="C134" s="366"/>
@@ -16758,20 +16814,19 @@
     </row>
     <row r="136" spans="1:23" ht="13" x14ac:dyDescent="0.15">
       <c r="A136" s="236">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B136" s="220"/>
-      <c r="C136" s="288" t="s">
-        <v>349</v>
+      <c r="C136" s="288" t="inlineStr">
+        <is>
+          <t>Annual Investment Allowance</t>
+        </is>
       </c>
       <c r="D136" s="227"/>
       <c r="E136" s="227"/>
       <c r="F136" s="227"/>
       <c r="G136" s="227"/>
-      <c r="H136" s="379">
-        <f>Admin!G4</f>
-        <v>1</v>
-      </c>
+      <c r="H136" s="379"/>
       <c r="I136" s="380"/>
       <c r="J136" s="227"/>
       <c r="K136" s="227"/>
@@ -16779,8 +16834,10 @@
         <v>54</v>
       </c>
       <c r="M136" s="220"/>
-      <c r="N136" s="227" t="s">
-        <v>223</v>
+      <c r="N136" s="227" t="inlineStr">
+        <is>
+          <t>Electric charge-point allowance</t>
+        </is>
       </c>
       <c r="O136" s="220"/>
       <c r="P136" s="220"/>
@@ -16806,9 +16863,7 @@
       <c r="K137" s="227"/>
       <c r="L137" s="227"/>
       <c r="M137" s="220"/>
-      <c r="N137" s="246" t="s">
-        <v>353</v>
-      </c>
+      <c r="N137" s="246"/>
       <c r="O137" s="258"/>
       <c r="P137" s="258"/>
       <c r="Q137" s="258"/>
@@ -16872,10 +16927,7 @@
       <c r="N139" s="217" t="s">
         <v>51</v>
       </c>
-      <c r="O139" s="356">
-        <f>IF(([1]Schedule!$R$1+[1]Schedule!$S$1)&lt;1000,[1]Schedule!$S$1,0)</f>
-        <v>0</v>
-      </c>
+      <c r="O139" s="356"/>
       <c r="P139" s="357"/>
       <c r="Q139" s="358"/>
       <c r="R139" s="218" t="s">
@@ -16918,11 +16970,13 @@
     </row>
     <row r="141" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A141" s="236">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B141" s="220"/>
-      <c r="C141" s="227" t="s">
-        <v>221</v>
+      <c r="C141" s="227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Capital allowances at </t>
+        </is>
       </c>
       <c r="D141" s="227"/>
       <c r="E141" s="227"/>
@@ -16932,8 +16986,10 @@
         <v>0.18</v>
       </c>
       <c r="H141" s="381"/>
-      <c r="I141" s="227" t="s">
-        <v>222</v>
+      <c r="I141" s="227" t="inlineStr">
+        <is>
+          <t>on equipment, including cars with lower CO2</t>
+        </is>
       </c>
       <c r="J141" s="227"/>
       <c r="K141" s="227"/>
@@ -16941,8 +16997,10 @@
         <v>55</v>
       </c>
       <c r="M141" s="220"/>
-      <c r="N141" s="227" t="s">
-        <v>225</v>
+      <c r="N141" s="227" t="inlineStr">
+        <is>
+          <t>100% and other enhanced capital allowances</t>
+        </is>
       </c>
       <c r="O141" s="220"/>
       <c r="P141" s="220"/>
@@ -16957,8 +17015,10 @@
     <row r="142" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A142" s="255"/>
       <c r="B142" s="220"/>
-      <c r="C142" s="227" t="s">
-        <v>224</v>
+      <c r="C142" s="227" t="inlineStr">
+        <is>
+          <t>emissions</t>
+        </is>
       </c>
       <c r="D142" s="227"/>
       <c r="E142" s="227"/>
@@ -16970,9 +17030,7 @@
       <c r="K142" s="227"/>
       <c r="L142" s="227"/>
       <c r="M142" s="220"/>
-      <c r="N142" s="227" t="s">
-        <v>226</v>
-      </c>
+      <c r="N142" s="227"/>
       <c r="O142" s="220"/>
       <c r="P142" s="220"/>
       <c r="Q142" s="220"/>
@@ -17015,7 +17073,7 @@
         <v>51</v>
       </c>
       <c r="D144" s="356">
-        <f>[1]Schedule!$R$1-D152</f>
+        <f>[1]Schedule!$R$1</f>
         <v>0</v>
       </c>
       <c r="E144" s="357"/>
@@ -17037,7 +17095,7 @@
         <v>51</v>
       </c>
       <c r="O144" s="356">
-        <f>[1]Schedule!$Y$1</f>
+        <f>IF(([1]Schedule!$R$1+[1]Schedule!$S$1)&lt;1000,[1]Schedule!$S$1,0)</f>
         <v>0</v>
       </c>
       <c r="P144" s="357"/>
@@ -17082,19 +17140,19 @@
     </row>
     <row r="146" spans="1:23" ht="13" x14ac:dyDescent="0.15">
       <c r="A146" s="236">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B146" s="220"/>
-      <c r="C146" s="288" t="s">
-        <v>354</v>
+      <c r="C146" s="288" t="inlineStr">
+        <is>
+          <t>Capital allowances at 6% on equipment, including cars with higher CO2 emissions</t>
+        </is>
       </c>
       <c r="D146" s="227"/>
       <c r="E146" s="227"/>
       <c r="F146" s="227"/>
       <c r="G146" s="227"/>
-      <c r="H146" s="379">
-        <v>0.1</v>
-      </c>
+      <c r="H146" s="379"/>
       <c r="I146" s="380"/>
       <c r="J146" s="220"/>
       <c r="K146" s="220"/>
@@ -17135,8 +17193,10 @@
         <v>56</v>
       </c>
       <c r="M147" s="220"/>
-      <c r="N147" s="227" t="s">
-        <v>355</v>
+      <c r="N147" s="227" t="inlineStr">
+        <is>
+          <t>Allowances on sale or cessation of business use (where you</t>
+        </is>
       </c>
       <c r="O147" s="220"/>
       <c r="P147" s="220"/>
@@ -17162,7 +17222,11 @@
       <c r="K148" s="220"/>
       <c r="L148" s="227"/>
       <c r="M148" s="220"/>
-      <c r="N148" s="220"/>
+      <c r="N148" s="227" t="inlineStr">
+        <is>
+          <t>have disposed of assets for less than their tax value)</t>
+        </is>
+      </c>
       <c r="O148" s="220"/>
       <c r="P148" s="220"/>
       <c r="Q148" s="220"/>
@@ -17175,11 +17239,13 @@
     </row>
     <row r="149" spans="1:23" ht="16" x14ac:dyDescent="0.15">
       <c r="A149" s="236">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B149" s="220"/>
-      <c r="C149" s="227" t="s">
-        <v>227</v>
+      <c r="C149" s="227" t="inlineStr">
+        <is>
+          <t>Zero-emission goods vehicle allowance</t>
+        </is>
       </c>
       <c r="D149" s="227"/>
       <c r="E149" s="227"/>
@@ -17195,7 +17261,7 @@
         <v>51</v>
       </c>
       <c r="O149" s="356">
-        <f>D139+D144+D147+D152+D156+D160+O139+O144</f>
+        <f>[1]Schedule!$Y$1</f>
         <v>0</v>
       </c>
       <c r="P149" s="357"/>
@@ -17216,9 +17282,7 @@
     <row r="150" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A150" s="240"/>
       <c r="B150" s="220"/>
-      <c r="C150" s="227" t="s">
-        <v>228</v>
-      </c>
+      <c r="C150" s="227"/>
       <c r="D150" s="220"/>
       <c r="E150" s="220"/>
       <c r="F150" s="220"/>
@@ -17256,8 +17320,10 @@
         <v>57</v>
       </c>
       <c r="M151" s="220"/>
-      <c r="N151" s="227" t="s">
-        <v>230</v>
+      <c r="N151" s="227" t="inlineStr">
+        <is>
+          <t>Total capital allowances (total of boxes 49 to 56)</t>
+        </is>
       </c>
       <c r="O151" s="220"/>
       <c r="P151" s="220"/>
@@ -17275,10 +17341,7 @@
       <c r="C152" s="217" t="s">
         <v>51</v>
       </c>
-      <c r="D152" s="356">
-        <f>SUM([1]Schedule!$R$38:$R$42)+SUM([1]Schedule!$R$91:$R$95)</f>
-        <v>0</v>
-      </c>
+      <c r="D152" s="356"/>
       <c r="E152" s="331"/>
       <c r="F152" s="332"/>
       <c r="G152" s="218" t="s">
@@ -17294,9 +17357,7 @@
       <c r="K152" s="220"/>
       <c r="L152" s="220"/>
       <c r="M152" s="220"/>
-      <c r="N152" s="227" t="s">
-        <v>231</v>
-      </c>
+      <c r="N152" s="227"/>
       <c r="O152" s="220"/>
       <c r="P152" s="220"/>
       <c r="Q152" s="220"/>
@@ -17334,11 +17395,13 @@
     </row>
     <row r="154" spans="1:23" ht="16" x14ac:dyDescent="0.15">
       <c r="A154" s="236">
-        <v>52</v>
+        <v>52.1</v>
       </c>
       <c r="B154" s="220"/>
-      <c r="C154" s="227" t="s">
-        <v>229</v>
+      <c r="C154" s="227" t="inlineStr">
+        <is>
+          <t>Zero-emission car allowance</t>
+        </is>
       </c>
       <c r="D154" s="227"/>
       <c r="E154" s="227"/>
@@ -17353,7 +17416,10 @@
       <c r="N154" s="217" t="s">
         <v>51</v>
       </c>
-      <c r="O154" s="356"/>
+      <c r="O154" s="356">
+        <f>D139+D144+D147+D152+D156+D160+O139+O144+O149</f>
+        <v>0</v>
+      </c>
       <c r="P154" s="357"/>
       <c r="Q154" s="358"/>
       <c r="R154" s="218" t="s">
@@ -17415,11 +17481,13 @@
       <c r="J156" s="220"/>
       <c r="K156" s="220"/>
       <c r="L156" s="236">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M156" s="220"/>
-      <c r="N156" s="227" t="s">
-        <v>356</v>
+      <c r="N156" s="227" t="inlineStr">
+        <is>
+          <t>Balancing charge on sales of assets or on the cessation of</t>
+        </is>
       </c>
       <c r="O156" s="220"/>
       <c r="P156" s="220"/>
@@ -17436,8 +17504,10 @@
         <v>53</v>
       </c>
       <c r="B157" s="220"/>
-      <c r="C157" s="227" t="s">
-        <v>232</v>
+      <c r="C157" s="227" t="inlineStr">
+        <is>
+          <t>The Structures and Buildings Allowance</t>
+        </is>
       </c>
       <c r="D157" s="227"/>
       <c r="E157" s="227"/>
@@ -17449,8 +17519,10 @@
       <c r="K157" s="227"/>
       <c r="L157" s="220"/>
       <c r="M157" s="220"/>
-      <c r="N157" s="227" t="s">
-        <v>357</v>
+      <c r="N157" s="227" t="inlineStr">
+        <is>
+          <t>business use (including where Business Premises Renovation</t>
+        </is>
       </c>
       <c r="O157" s="220"/>
       <c r="P157" s="220"/>
@@ -17465,9 +17537,7 @@
     <row r="158" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A158" s="240"/>
       <c r="B158" s="220"/>
-      <c r="C158" s="227" t="s">
-        <v>358</v>
-      </c>
+      <c r="C158" s="227"/>
       <c r="D158" s="220"/>
       <c r="E158" s="220"/>
       <c r="F158" s="220"/>
@@ -17478,8 +17548,10 @@
       <c r="K158" s="220"/>
       <c r="L158" s="220"/>
       <c r="M158" s="220"/>
-      <c r="N158" s="227" t="s">
-        <v>359</v>
+      <c r="N158" s="227" t="inlineStr">
+        <is>
+          <t>Allowance has been claimed)</t>
+        </is>
       </c>
       <c r="O158" s="220"/>
       <c r="P158" s="220"/>
@@ -17613,8 +17685,10 @@
       <c r="W162" s="365"/>
     </row>
     <row r="163" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A163" s="366" t="s">
-        <v>234</v>
+      <c r="A163" s="366" t="inlineStr">
+        <is>
+          <t>You may have to adjust your net profit or loss for disallowable expenses or capital allowances to arrive at your taxable profit</t>
+        </is>
       </c>
       <c r="B163" s="366"/>
       <c r="C163" s="366"/>
@@ -17640,8 +17714,10 @@
       <c r="W163" s="366"/>
     </row>
     <row r="164" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A164" s="366" t="s">
-        <v>360</v>
+      <c r="A164" s="366" t="inlineStr">
+        <is>
+          <t>or your loss for tax purposes. Please read the 'Self-employment (full) notes' and fill in the boxes below that apply.</t>
+        </is>
       </c>
       <c r="B164" s="366"/>
       <c r="C164" s="366"/>
@@ -17693,11 +17769,13 @@
     </row>
     <row r="166" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A166" s="236">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B166" s="220"/>
-      <c r="C166" s="227" t="s">
-        <v>361</v>
+      <c r="C166" s="227" t="inlineStr">
+        <is>
+          <t>Goods and services for your own use</t>
+        </is>
       </c>
       <c r="D166" s="227"/>
       <c r="E166" s="227"/>
@@ -17708,7 +17786,7 @@
       <c r="J166" s="227"/>
       <c r="K166" s="227"/>
       <c r="L166" s="236">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M166" s="220"/>
       <c r="N166" s="227" t="s">
@@ -17727,9 +17805,7 @@
     <row r="167" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A167" s="255"/>
       <c r="B167" s="220"/>
-      <c r="C167" s="227" t="s">
-        <v>236</v>
-      </c>
+      <c r="C167" s="227"/>
       <c r="D167" s="227"/>
       <c r="E167" s="227"/>
       <c r="F167" s="227"/>
@@ -17740,8 +17816,10 @@
       <c r="K167" s="227"/>
       <c r="L167" s="227"/>
       <c r="M167" s="220"/>
-      <c r="N167" s="227" t="s">
-        <v>362</v>
+      <c r="N167" s="227" t="inlineStr">
+        <is>
+          <t>net loss (box 57 + box 62)</t>
+        </is>
       </c>
       <c r="O167" s="258"/>
       <c r="P167" s="258"/>
@@ -17807,7 +17885,7 @@
         <v>51</v>
       </c>
       <c r="O169" s="356">
-        <f>O149+D179</f>
+        <f>O154+D179</f>
         <v>0</v>
       </c>
       <c r="P169" s="357"/>
@@ -17852,7 +17930,7 @@
     </row>
     <row r="171" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A171" s="236">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B171" s="220"/>
       <c r="C171" s="227" t="s">
@@ -17867,11 +17945,13 @@
       <c r="J171" s="227"/>
       <c r="K171" s="227"/>
       <c r="L171" s="236">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M171" s="220"/>
-      <c r="N171" s="227" t="s">
-        <v>363</v>
+      <c r="N171" s="227" t="inlineStr">
+        <is>
+          <t>Net business profit for tax purposes (if box 47 + box 61</t>
+        </is>
       </c>
       <c r="O171" s="220"/>
       <c r="P171" s="220"/>
@@ -17886,8 +17966,10 @@
     <row r="172" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A172" s="255"/>
       <c r="B172" s="220"/>
-      <c r="C172" s="227" t="s">
-        <v>364</v>
+      <c r="C172" s="227" t="inlineStr">
+        <is>
+          <t>(box 46 + box 59 + box 60)</t>
+        </is>
       </c>
       <c r="D172" s="227"/>
       <c r="E172" s="227"/>
@@ -17899,8 +17981,10 @@
       <c r="K172" s="227"/>
       <c r="L172" s="227"/>
       <c r="M172" s="220"/>
-      <c r="N172" s="227" t="s">
-        <v>365</v>
+      <c r="N172" s="227" t="inlineStr">
+        <is>
+          <t>minus (box 48 + box 63) is positive)</t>
+        </is>
       </c>
       <c r="O172" s="220"/>
       <c r="P172" s="220"/>
@@ -17944,7 +18028,7 @@
         <v>51</v>
       </c>
       <c r="D174" s="356">
-        <f>O122+O154+O160+D169</f>
+        <f>O122+O160+D169</f>
         <v>0</v>
       </c>
       <c r="E174" s="357"/>
@@ -18011,7 +18095,7 @@
     </row>
     <row r="176" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A176" s="236">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B176" s="220"/>
       <c r="C176" s="227" t="s">
@@ -18026,11 +18110,13 @@
       <c r="J176" s="227"/>
       <c r="K176" s="227"/>
       <c r="L176" s="236">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="M176" s="220"/>
-      <c r="N176" s="227" t="s">
-        <v>366</v>
+      <c r="N176" s="227" t="inlineStr">
+        <is>
+          <t>Net business loss for tax purposes (if box 48 + box 63</t>
+        </is>
       </c>
       <c r="O176" s="220"/>
       <c r="P176" s="220"/>
@@ -18058,8 +18144,10 @@
       <c r="K177" s="220"/>
       <c r="L177" s="220"/>
       <c r="M177" s="220"/>
-      <c r="N177" s="227" t="s">
-        <v>367</v>
+      <c r="N177" s="227" t="inlineStr">
+        <is>
+          <t>minus (box 47 + box 61) is positive)</t>
+        </is>
       </c>
       <c r="O177" s="220"/>
       <c r="P177" s="220"/>
@@ -18193,8 +18281,10 @@
       <c r="W181" s="365"/>
     </row>
     <row r="182" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A182" s="366" t="s">
-        <v>241</v>
+      <c r="A182" s="366" t="inlineStr">
+        <is>
+          <t>Please read the 'Self-employment (full) notes' and fill in the boxes below that apply. If your accounting date is not between</t>
+        </is>
       </c>
       <c r="B182" s="366"/>
       <c r="C182" s="366"/>
@@ -18220,8 +18310,10 @@
       <c r="W182" s="366"/>
     </row>
     <row r="183" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A183" s="366" t="s">
-        <v>242</v>
+      <c r="A183" s="366" t="inlineStr">
+        <is>
+          <t>31 March and 5 April you will need to apportion profits from each accounting period to the tax year - use box 68 to adjust</t>
+        </is>
       </c>
       <c r="B183" s="366"/>
       <c r="C183" s="366"/>
@@ -18247,8 +18339,10 @@
       <c r="W183" s="366"/>
     </row>
     <row r="184" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A184" s="387" t="s">
-        <v>243</v>
+      <c r="A184" s="387" t="inlineStr">
+        <is>
+          <t>your tax profit (box 64) or loss (box 65) accordingly.</t>
+        </is>
       </c>
       <c r="B184" s="387"/>
       <c r="C184" s="387"/>
@@ -18299,12 +18393,12 @@
       <c r="W185" s="235"/>
     </row>
     <row r="186" spans="1:23" x14ac:dyDescent="0.15">
-      <c r="A186" s="236">
-        <v>65</v>
-      </c>
+      <c r="A186" s="236"/>
       <c r="B186" s="220"/>
-      <c r="C186" s="227" t="s">
-        <v>244</v>
+      <c r="C186" s="227" t="inlineStr">
+        <is>
+          <t>Boxes 66 and 67 are not in use</t>
+        </is>
       </c>
       <c r="D186" s="227"/>
       <c r="E186" s="227"/>
@@ -18315,7 +18409,7 @@
       <c r="J186" s="227"/>
       <c r="K186" s="227"/>
       <c r="L186" s="236">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="M186" s="220"/>
       <c r="N186" s="227" t="s">
@@ -18372,8 +18466,10 @@
       <c r="K188" s="220"/>
       <c r="L188" s="227"/>
       <c r="M188" s="220"/>
-      <c r="N188" s="248" t="s">
-        <v>247</v>
+      <c r="N188" s="248" t="inlineStr">
+        <is>
+          <t>adjustment needs to be taken off the profit figure, put a</t>
+        </is>
       </c>
       <c r="O188" s="220"/>
       <c r="P188" s="220"/>
@@ -18386,13 +18482,9 @@
       <c r="W188" s="243"/>
     </row>
     <row r="189" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A189" s="236">
-        <v>66</v>
-      </c>
+      <c r="A189" s="236"/>
       <c r="B189" s="220"/>
-      <c r="C189" s="227" t="s">
-        <v>248</v>
-      </c>
+      <c r="C189" s="227"/>
       <c r="D189" s="220"/>
       <c r="E189" s="220"/>
       <c r="F189" s="220"/>
@@ -18478,11 +18570,13 @@
     </row>
     <row r="192" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A192" s="236">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B192" s="220"/>
-      <c r="C192" s="227" t="s">
-        <v>251</v>
+      <c r="C192" s="227" t="inlineStr">
+        <is>
+          <t>Adjustment where your accounting period was not 12 months</t>
+        </is>
       </c>
       <c r="D192" s="259"/>
       <c r="E192" s="259"/>
@@ -18493,11 +18587,13 @@
       <c r="J192" s="220"/>
       <c r="K192" s="220"/>
       <c r="L192" s="236">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M192" s="220"/>
-      <c r="N192" s="227" t="s">
-        <v>252</v>
+      <c r="N192" s="227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adjusted profit for </t>
+        </is>
       </c>
       <c r="O192" s="220"/>
       <c r="P192" s="220"/>
@@ -18505,9 +18601,7 @@
         <f>Admin!G2</f>
         <v>2025-26</v>
       </c>
-      <c r="R192" s="227" t="s">
-        <v>368</v>
-      </c>
+      <c r="R192" s="227"/>
       <c r="S192" s="220"/>
       <c r="T192" s="220"/>
       <c r="U192" s="220"/>
@@ -18517,8 +18611,10 @@
     <row r="193" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A193" s="240"/>
       <c r="B193" s="220"/>
-      <c r="C193" s="227" t="s">
-        <v>253</v>
+      <c r="C193" s="227" t="inlineStr">
+        <is>
+          <t>long or ended before 31 March - if the adjustment needs to be</t>
+        </is>
       </c>
       <c r="D193" s="227"/>
       <c r="E193" s="227"/>
@@ -18530,8 +18626,10 @@
       <c r="K193" s="227"/>
       <c r="L193" s="227"/>
       <c r="M193" s="227"/>
-      <c r="N193" s="241" t="s">
-        <v>369</v>
+      <c r="N193" s="241" t="inlineStr">
+        <is>
+          <t>- see the working sheet in the notes</t>
+        </is>
       </c>
       <c r="O193" s="259"/>
       <c r="P193" s="259"/>
@@ -18546,8 +18644,10 @@
     <row r="194" spans="1:23" ht="16" x14ac:dyDescent="0.15">
       <c r="A194" s="240"/>
       <c r="B194" s="220"/>
-      <c r="C194" s="241" t="s">
-        <v>254</v>
+      <c r="C194" s="241" t="inlineStr">
+        <is>
+          <t>taken off the profit figure, put a minus sign (-) in the box</t>
+        </is>
       </c>
       <c r="D194" s="227"/>
       <c r="E194" s="227"/>
@@ -18584,9 +18684,7 @@
     <row r="195" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A195" s="240"/>
       <c r="B195" s="220"/>
-      <c r="C195" s="227" t="s">
-        <v>255</v>
-      </c>
+      <c r="C195" s="227"/>
       <c r="D195" s="220"/>
       <c r="E195" s="220"/>
       <c r="F195" s="220"/>
@@ -18611,9 +18709,7 @@
     <row r="196" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A196" s="255"/>
       <c r="B196" s="220"/>
-      <c r="C196" s="227" t="s">
-        <v>256</v>
-      </c>
+      <c r="C196" s="227"/>
       <c r="D196" s="227"/>
       <c r="E196" s="227"/>
       <c r="F196" s="227"/>
@@ -18623,11 +18719,13 @@
       <c r="J196" s="227"/>
       <c r="K196" s="227"/>
       <c r="L196" s="236">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M196" s="220"/>
-      <c r="N196" s="227" t="s">
-        <v>257</v>
+      <c r="N196" s="227" t="inlineStr">
+        <is>
+          <t>Loss brought forward from earlier years set off against</t>
+        </is>
       </c>
       <c r="O196" s="220"/>
       <c r="P196" s="220"/>
@@ -18663,8 +18761,10 @@
       <c r="K197" s="220"/>
       <c r="L197" s="220"/>
       <c r="M197" s="220"/>
-      <c r="N197" s="241" t="s">
-        <v>370</v>
+      <c r="N197" s="241" t="inlineStr">
+        <is>
+          <t>this year's adjusted profit</t>
+        </is>
       </c>
       <c r="O197" s="220"/>
       <c r="P197" s="220"/>
@@ -18690,9 +18790,7 @@
       <c r="K198" s="220"/>
       <c r="L198" s="220"/>
       <c r="M198" s="220"/>
-      <c r="N198" s="246" t="s">
-        <v>371</v>
-      </c>
+      <c r="N198" s="246"/>
       <c r="O198" s="220"/>
       <c r="P198" s="220"/>
       <c r="Q198" s="220"/>
@@ -18704,12 +18802,12 @@
       <c r="W198" s="243"/>
     </row>
     <row r="199" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A199" s="236">
-        <v>68</v>
-      </c>
+      <c r="A199" s="236"/>
       <c r="B199" s="220"/>
-      <c r="C199" s="227" t="s">
-        <v>372</v>
+      <c r="C199" s="227" t="inlineStr">
+        <is>
+          <t>Boxes 69 and 70 are not in use</t>
+        </is>
       </c>
       <c r="D199" s="220"/>
       <c r="E199" s="220"/>
@@ -18771,29 +18869,23 @@
     <row r="201" spans="1:23" ht="16" x14ac:dyDescent="0.15">
       <c r="A201" s="240"/>
       <c r="B201" s="220"/>
-      <c r="C201" s="217" t="s">
-        <v>51</v>
-      </c>
+      <c r="C201" s="217"/>
       <c r="D201" s="356"/>
       <c r="E201" s="357"/>
       <c r="F201" s="358"/>
-      <c r="G201" s="218" t="s">
-        <v>178</v>
-      </c>
-      <c r="H201" s="219">
-        <v>0</v>
-      </c>
-      <c r="I201" s="219">
-        <v>0</v>
-      </c>
+      <c r="G201" s="218"/>
+      <c r="H201" s="219"/>
+      <c r="I201" s="219"/>
       <c r="J201" s="220"/>
       <c r="K201" s="220"/>
       <c r="L201" s="236">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M201" s="220"/>
-      <c r="N201" s="227" t="s">
-        <v>258</v>
+      <c r="N201" s="227" t="inlineStr">
+        <is>
+          <t>Any other business income not included in</t>
+        </is>
       </c>
       <c r="O201" s="220"/>
       <c r="P201" s="220"/>
@@ -18819,8 +18911,10 @@
       <c r="K202" s="220"/>
       <c r="L202" s="220"/>
       <c r="M202" s="220"/>
-      <c r="N202" s="227" t="s">
-        <v>373</v>
+      <c r="N202" s="227" t="inlineStr">
+        <is>
+          <t>boxes 15, 16 or 60</t>
+        </is>
       </c>
       <c r="O202" s="220"/>
       <c r="P202" s="220"/>
@@ -18833,13 +18927,9 @@
       <c r="W202" s="243"/>
     </row>
     <row r="203" spans="1:23" x14ac:dyDescent="0.15">
-      <c r="A203" s="236">
-        <v>69</v>
-      </c>
+      <c r="A203" s="236"/>
       <c r="B203" s="220"/>
-      <c r="C203" s="227" t="s">
-        <v>374</v>
-      </c>
+      <c r="C203" s="227"/>
       <c r="D203" s="227"/>
       <c r="E203" s="227"/>
       <c r="F203" s="227"/>
@@ -18925,29 +19015,23 @@
     <row r="206" spans="1:23" ht="16" x14ac:dyDescent="0.15">
       <c r="A206" s="240"/>
       <c r="B206" s="220"/>
-      <c r="C206" s="217" t="s">
-        <v>51</v>
-      </c>
+      <c r="C206" s="217"/>
       <c r="D206" s="356"/>
       <c r="E206" s="357"/>
       <c r="F206" s="358"/>
-      <c r="G206" s="218" t="s">
-        <v>178</v>
-      </c>
-      <c r="H206" s="219">
-        <v>0</v>
-      </c>
-      <c r="I206" s="219">
-        <v>0</v>
-      </c>
+      <c r="G206" s="218"/>
+      <c r="H206" s="219"/>
+      <c r="I206" s="219"/>
       <c r="J206" s="220"/>
       <c r="K206" s="220"/>
       <c r="L206" s="236">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="M206" s="220"/>
-      <c r="N206" s="227" t="s">
-        <v>375</v>
+      <c r="N206" s="227" t="inlineStr">
+        <is>
+          <t>Total taxable profits from this business</t>
+        </is>
       </c>
       <c r="O206" s="220"/>
       <c r="P206" s="220"/>
@@ -18973,8 +19057,10 @@
       <c r="K207" s="220"/>
       <c r="L207" s="220"/>
       <c r="M207" s="220"/>
-      <c r="N207" s="227" t="s">
-        <v>376</v>
+      <c r="N207" s="227" t="inlineStr">
+        <is>
+          <t>- see the working sheet in the notes</t>
+        </is>
       </c>
       <c r="O207" s="220"/>
       <c r="P207" s="220"/>
@@ -18988,11 +19074,13 @@
     </row>
     <row r="208" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A208" s="236">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B208" s="220"/>
-      <c r="C208" s="227" t="s">
-        <v>259</v>
+      <c r="C208" s="227" t="inlineStr">
+        <is>
+          <t>Adjustment for change of accounting practice</t>
+        </is>
       </c>
       <c r="D208" s="227"/>
       <c r="E208" s="227"/>
@@ -19004,9 +19092,7 @@
       <c r="K208" s="227"/>
       <c r="L208" s="220"/>
       <c r="M208" s="220"/>
-      <c r="N208" s="246" t="s">
-        <v>377</v>
-      </c>
+      <c r="N208" s="246"/>
       <c r="O208" s="220"/>
       <c r="P208" s="220"/>
       <c r="Q208" s="220"/>
@@ -19020,9 +19106,7 @@
     <row r="209" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A209" s="240"/>
       <c r="B209" s="220"/>
-      <c r="C209" s="248" t="s">
-        <v>378</v>
-      </c>
+      <c r="C209" s="248"/>
       <c r="D209" s="220"/>
       <c r="E209" s="220"/>
       <c r="F209" s="220"/>
@@ -19141,8 +19225,10 @@
       <c r="W212" s="368"/>
     </row>
     <row r="213" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A213" s="366" t="s">
-        <v>261</v>
+      <c r="A213" s="366" t="inlineStr">
+        <is>
+          <t>If you have made a net loss for tax purposes (in box 65), or because of box 68, or if you have losses from previous years,</t>
+        </is>
       </c>
       <c r="B213" s="366"/>
       <c r="C213" s="366"/>
@@ -19168,8 +19254,10 @@
       <c r="W213" s="366"/>
     </row>
     <row r="214" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A214" s="366" t="s">
-        <v>262</v>
+      <c r="A214" s="366" t="inlineStr">
+        <is>
+          <t>read the 'Self-employment (full) notes' and fill in boxes 77 to 80 as appropriate.</t>
+        </is>
       </c>
       <c r="B214" s="366"/>
       <c r="C214" s="366"/>
@@ -19221,11 +19309,13 @@
     </row>
     <row r="216" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A216" s="236">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B216" s="220"/>
-      <c r="C216" s="227" t="s">
-        <v>263</v>
+      <c r="C216" s="227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adjusted loss for </t>
+        </is>
       </c>
       <c r="D216" s="227"/>
       <c r="E216" s="227"/>
@@ -19233,15 +19323,17 @@
         <f>Admin!G2</f>
         <v>2025-26</v>
       </c>
-      <c r="G216" s="227" t="s">
-        <v>379</v>
+      <c r="G216" s="227" t="inlineStr">
+        <is>
+          <t>- see the working sheet in the notes</t>
+        </is>
       </c>
       <c r="H216" s="227"/>
       <c r="I216" s="227"/>
       <c r="J216" s="220"/>
       <c r="K216" s="227"/>
       <c r="L216" s="236">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="M216" s="220"/>
       <c r="N216" s="227" t="s">
@@ -19260,9 +19352,7 @@
     <row r="217" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A217" s="255"/>
       <c r="B217" s="220"/>
-      <c r="C217" s="227" t="s">
-        <v>380</v>
-      </c>
+      <c r="C217" s="227"/>
       <c r="D217" s="227"/>
       <c r="E217" s="227"/>
       <c r="F217" s="227"/>
@@ -19318,7 +19408,7 @@
         <v>51</v>
       </c>
       <c r="D219" s="356">
-        <f>O179+E197-D201+D210+P190</f>
+        <f>O179+E197+D210+P190</f>
         <v>0</v>
       </c>
       <c r="E219" s="357"/>
@@ -19382,7 +19472,7 @@
     </row>
     <row r="221" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A221" s="236">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B221" s="220"/>
       <c r="C221" s="227" t="s">
@@ -19397,7 +19487,7 @@
       <c r="J221" s="227"/>
       <c r="K221" s="227"/>
       <c r="L221" s="236">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="M221" s="220"/>
       <c r="N221" s="227" t="s">
@@ -19540,8 +19630,10 @@
       <c r="W225" s="251"/>
     </row>
     <row r="226" spans="1:23" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A226" s="388" t="s">
-        <v>270</v>
+      <c r="A226" s="388" t="inlineStr">
+        <is>
+          <t>CIS deductions and tax taken off</t>
+        </is>
       </c>
       <c r="B226" s="388"/>
       <c r="C226" s="388"/>
@@ -19593,11 +19685,13 @@
     </row>
     <row r="228" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A228" s="236">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B228" s="220"/>
-      <c r="C228" s="227" t="s">
-        <v>271</v>
+      <c r="C228" s="227" t="inlineStr">
+        <is>
+          <t>Total Construction Industry Scheme (CIS) deductions taken from</t>
+        </is>
       </c>
       <c r="D228" s="227"/>
       <c r="E228" s="227"/>
@@ -19608,7 +19702,7 @@
       <c r="J228" s="227"/>
       <c r="K228" s="227"/>
       <c r="L228" s="236">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M228" s="220"/>
       <c r="N228" s="227" t="s">
@@ -19627,8 +19721,10 @@
     <row r="229" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A229" s="255"/>
       <c r="B229" s="220"/>
-      <c r="C229" s="227" t="s">
-        <v>273</v>
+      <c r="C229" s="227" t="inlineStr">
+        <is>
+          <t>your payments by contractors - CIS subcontractors only</t>
+        </is>
       </c>
       <c r="D229" s="227"/>
       <c r="E229" s="227"/>
@@ -19773,8 +19869,10 @@
       <c r="W233" s="365"/>
     </row>
     <row r="234" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A234" s="366" t="s">
-        <v>274</v>
+      <c r="A234" s="366" t="inlineStr">
+        <is>
+          <t>If your business accounts include a balance sheet showing the assets, liabilities and capital of the business, fill in the relevant</t>
+        </is>
       </c>
       <c r="B234" s="366"/>
       <c r="C234" s="366"/>
@@ -19800,8 +19898,10 @@
       <c r="W234" s="366"/>
     </row>
     <row r="235" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A235" s="366" t="s">
-        <v>382</v>
+      <c r="A235" s="366" t="inlineStr">
+        <is>
+          <t>boxes below. If you do not have a balance sheet, go to box 100.</t>
+        </is>
       </c>
       <c r="B235" s="366"/>
       <c r="C235" s="366"/>
@@ -19907,7 +20007,7 @@
     </row>
     <row r="239" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A239" s="236">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B239" s="220"/>
       <c r="C239" s="227" t="s">
@@ -19922,7 +20022,7 @@
       <c r="J239" s="227"/>
       <c r="K239" s="227"/>
       <c r="L239" s="236">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="M239" s="220"/>
       <c r="N239" s="227" t="s">
@@ -20031,7 +20131,7 @@
     </row>
     <row r="243" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A243" s="236">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B243" s="220"/>
       <c r="C243" s="227" t="s">
@@ -20046,7 +20146,7 @@
       <c r="J243" s="227"/>
       <c r="K243" s="227"/>
       <c r="L243" s="236">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="M243" s="220"/>
       <c r="N243" s="227" t="s">
@@ -20155,7 +20255,7 @@
     </row>
     <row r="247" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A247" s="236">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B247" s="220"/>
       <c r="C247" s="227" t="s">
@@ -20170,7 +20270,7 @@
       <c r="J247" s="227"/>
       <c r="K247" s="227"/>
       <c r="L247" s="236">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="M247" s="220"/>
       <c r="N247" s="227" t="s">
@@ -20279,7 +20379,7 @@
     </row>
     <row r="251" spans="1:23" ht="16" x14ac:dyDescent="0.15">
       <c r="A251" s="236">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B251" s="220"/>
       <c r="C251" s="227" t="s">
@@ -20354,11 +20454,13 @@
       <c r="J253" s="220"/>
       <c r="K253" s="220"/>
       <c r="L253" s="236">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="M253" s="220"/>
-      <c r="N253" s="227" t="s">
-        <v>285</v>
+      <c r="N253" s="227" t="inlineStr">
+        <is>
+          <t>Net business assets (box 90 minus (boxes 91 to 93))</t>
+        </is>
       </c>
       <c r="O253" s="220"/>
       <c r="P253" s="220"/>
@@ -20397,11 +20499,13 @@
     </row>
     <row r="255" spans="1:23" ht="16" x14ac:dyDescent="0.15">
       <c r="A255" s="236">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B255" s="220"/>
-      <c r="C255" s="227" t="s">
-        <v>286</v>
+      <c r="C255" s="227" t="inlineStr">
+        <is>
+          <t>Bank or building society balances</t>
+        </is>
       </c>
       <c r="D255" s="227"/>
       <c r="E255" s="227"/>
@@ -20521,7 +20625,7 @@
     </row>
     <row r="259" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A259" s="236">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B259" s="220"/>
       <c r="C259" s="227" t="s">
@@ -20536,7 +20640,7 @@
       <c r="J259" s="227"/>
       <c r="K259" s="227"/>
       <c r="L259" s="236">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M259" s="220"/>
       <c r="N259" s="227" t="s">
@@ -20647,7 +20751,7 @@
     </row>
     <row r="263" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A263" s="236">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B263" s="220"/>
       <c r="C263" s="227" t="s">
@@ -20662,11 +20766,13 @@
       <c r="J263" s="227"/>
       <c r="K263" s="227"/>
       <c r="L263" s="236">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M263" s="220"/>
-      <c r="N263" s="227" t="s">
-        <v>291</v>
+      <c r="N263" s="227" t="inlineStr">
+        <is>
+          <t>Net profit or loss (box 47 or box 48)</t>
+        </is>
       </c>
       <c r="O263" s="220"/>
       <c r="P263" s="220"/>
@@ -20773,11 +20879,13 @@
     </row>
     <row r="267" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A267" s="236">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B267" s="220"/>
-      <c r="C267" s="227" t="s">
-        <v>292</v>
+      <c r="C267" s="227" t="inlineStr">
+        <is>
+          <t>Total assets (total of boxes 83 to 89)</t>
+        </is>
       </c>
       <c r="D267" s="227"/>
       <c r="E267" s="227"/>
@@ -20788,7 +20896,7 @@
       <c r="J267" s="227"/>
       <c r="K267" s="227"/>
       <c r="L267" s="236">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="M267" s="220"/>
       <c r="N267" s="227" t="s">
@@ -20908,7 +21016,7 @@
       <c r="J271" s="227"/>
       <c r="K271" s="227"/>
       <c r="L271" s="236">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="M271" s="220"/>
       <c r="N271" s="227" t="s">
@@ -21020,7 +21128,7 @@
       <c r="J275" s="227"/>
       <c r="K275" s="227"/>
       <c r="L275" s="236">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M275" s="220"/>
       <c r="N275" s="227" t="s">
@@ -21122,8 +21230,10 @@
       <c r="W278" s="251"/>
     </row>
     <row r="279" spans="1:23" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A279" s="368" t="s">
-        <v>295</v>
+      <c r="A279" s="368" t="inlineStr">
+        <is>
+          <t>Class 2 and Class 4 National Insurance contributions (NICs)</t>
+        </is>
       </c>
       <c r="B279" s="368"/>
       <c r="C279" s="368"/>
@@ -21149,8 +21259,10 @@
       <c r="W279" s="368"/>
     </row>
     <row r="280" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A280" s="366" t="s">
-        <v>296</v>
+      <c r="A280" s="366" t="inlineStr">
+        <is>
+          <t>If your self employed profits are more than £</t>
+        </is>
       </c>
       <c r="B280" s="399"/>
       <c r="C280" s="399"/>
@@ -21161,11 +21273,13 @@
       <c r="H280" s="399"/>
       <c r="I280" s="399"/>
       <c r="J280" s="285">
-        <f>Admin!N4</f>
+        <f>Admin!N20</f>
         <v>12570</v>
       </c>
-      <c r="K280" s="366" t="s">
-        <v>297</v>
+      <c r="K280" s="366" t="inlineStr">
+        <is>
+          <t>you must pay Class 4 NICs (unless you are exempt) - read the notes.</t>
+        </is>
       </c>
       <c r="L280" s="346"/>
       <c r="M280" s="346"/>
@@ -21181,8 +21295,10 @@
       <c r="W280" s="346"/>
     </row>
     <row r="281" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A281" s="398" t="s">
-        <v>383</v>
+      <c r="A281" s="398" t="inlineStr">
+        <is>
+          <t>If your total profits are below the Class 2 small profits threshold you do not have to pay Class 2 NICs, but you may pay them voluntarily.</t>
+        </is>
       </c>
       <c r="B281" s="398"/>
       <c r="C281" s="398"/>
@@ -21234,11 +21350,13 @@
     </row>
     <row r="283" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A283" s="236">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B283" s="220"/>
-      <c r="C283" s="227" t="s">
-        <v>298</v>
+      <c r="C283" s="227" t="inlineStr">
+        <is>
+          <t>If your total profits are below the Class 2 small profits threshold</t>
+        </is>
       </c>
       <c r="D283" s="220"/>
       <c r="E283" s="220"/>
@@ -21249,7 +21367,7 @@
       <c r="J283" s="220"/>
       <c r="K283" s="220"/>
       <c r="L283" s="236">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M283" s="220"/>
       <c r="N283" s="227" t="s">
@@ -21268,8 +21386,10 @@
     <row r="284" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A284" s="240"/>
       <c r="B284" s="220"/>
-      <c r="C284" s="227" t="s">
-        <v>384</v>
+      <c r="C284" s="227" t="inlineStr">
+        <is>
+          <t>and you choose to pay Class 2 NICs voluntarily, put 'X' in the box</t>
+        </is>
       </c>
       <c r="D284" s="220"/>
       <c r="E284" s="220"/>
@@ -21379,24 +21499,21 @@
     </row>
     <row r="288" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A288" s="236">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B288" s="220"/>
-      <c r="C288" s="227" t="s">
-        <v>301</v>
+      <c r="C288" s="227" t="inlineStr">
+        <is>
+          <t>If you are exempt from paying Class 4 NICs, put 'X' in the box</t>
+        </is>
       </c>
       <c r="D288" s="220"/>
       <c r="E288" s="220"/>
       <c r="F288" s="220"/>
-      <c r="G288" s="370" t="str">
-        <f>Admin!G2</f>
-        <v>2025-26</v>
-      </c>
+      <c r="G288" s="370"/>
       <c r="H288" s="371"/>
       <c r="I288" s="371"/>
-      <c r="J288" s="220" t="s">
-        <v>302</v>
-      </c>
+      <c r="J288" s="220"/>
       <c r="K288" s="220"/>
       <c r="L288" s="220"/>
       <c r="M288" s="220"/>
@@ -21414,8 +21531,10 @@
     <row r="289" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A289" s="240"/>
       <c r="B289" s="220"/>
-      <c r="C289" s="227" t="s">
-        <v>385</v>
+      <c r="C289" s="227" t="inlineStr">
+        <is>
+          <t>- read the notes</t>
+        </is>
       </c>
       <c r="D289" s="220"/>
       <c r="E289" s="220"/>
@@ -21441,9 +21560,7 @@
     <row r="290" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A290" s="240"/>
       <c r="B290" s="220"/>
-      <c r="C290" s="220" t="s">
-        <v>303</v>
-      </c>
+      <c r="C290" s="220"/>
       <c r="D290" s="220"/>
       <c r="E290" s="220"/>
       <c r="F290" s="220"/>
@@ -21594,11 +21711,13 @@
     </row>
     <row r="296" spans="1:23" x14ac:dyDescent="0.15">
       <c r="A296" s="236">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B296" s="220"/>
-      <c r="C296" s="227" t="s">
-        <v>305</v>
+      <c r="C296" s="227" t="inlineStr">
+        <is>
+          <t>Please give any other information in this space</t>
+        </is>
       </c>
       <c r="D296" s="220"/>
       <c r="E296" s="220"/>

</xml_diff>